<commit_message>
Complete indicadores module: monthly & quarterly views, semaphore, area stats
</commit_message>
<xml_diff>
--- a/formatos/Cuadro de Control Marzo 2026.xlsx
+++ b/formatos/Cuadro de Control Marzo 2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/530d8857ba2bb3e5/Favorites/Escritorio/SGC page/formatos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="363" documentId="8_{F0B4F5C4-B2C8-463D-A3E4-1B22D6C2B5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD38E923-EDDC-4BC0-A5B2-69E8877F154D}"/>
+  <xr:revisionPtr revIDLastSave="378" documentId="8_{F0B4F5C4-B2C8-463D-A3E4-1B22D6C2B5BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{775FDD25-E782-4274-949F-29D03C728F68}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="18696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1357" uniqueCount="463">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1576" uniqueCount="463">
   <si>
     <t>OOMRSC-05</t>
   </si>
@@ -3504,7 +3504,7 @@
   <dimension ref="A1:BA133"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="6.44140625" style="17" customWidth="1"/>
+    <col min="1" max="1" width="28.6640625" style="17" customWidth="1"/>
     <col min="2" max="2" width="29.5546875" style="17" customWidth="1"/>
     <col min="3" max="3" width="23.6640625" style="17" customWidth="1"/>
     <col min="4" max="4" width="33.6640625" style="17" customWidth="1"/>
@@ -3606,8 +3606,7 @@
       <c r="A2" s="23" t="s">
         <v>453</v>
       </c>
-      <c r="B2" s="148"/>
-      <c r="C2" s="63" t="s">
+      <c r="B2" s="63" t="s">
         <v>1</v>
       </c>
       <c r="D2" s="63"/>
@@ -3895,8 +3894,12 @@
     <row r="6" spans="1:53" s="1" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="252"/>
       <c r="B6" s="252"/>
-      <c r="C6" s="252"/>
-      <c r="D6" s="252"/>
+      <c r="C6" s="252" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="252" t="s">
+        <v>6</v>
+      </c>
       <c r="E6" s="252"/>
       <c r="F6" s="252"/>
       <c r="G6" s="252"/>
@@ -4148,8 +4151,12 @@
     </row>
     <row r="8" spans="1:53" s="2" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="77"/>
-      <c r="B8" s="37"/>
-      <c r="C8" s="214"/>
+      <c r="B8" s="37" t="s">
+        <v>55</v>
+      </c>
+      <c r="C8" s="214" t="s">
+        <v>56</v>
+      </c>
       <c r="D8" s="163" t="s">
         <v>63</v>
       </c>
@@ -4291,9 +4298,15 @@
     </row>
     <row r="9" spans="1:53" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="71"/>
-      <c r="B9" s="43"/>
-      <c r="C9" s="237"/>
-      <c r="D9" s="215"/>
+      <c r="B9" s="43" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" s="237" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" s="215" t="s">
+        <v>63</v>
+      </c>
       <c r="E9" s="64">
         <v>2</v>
       </c>
@@ -4581,9 +4594,15 @@
     </row>
     <row r="11" spans="1:53" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="35"/>
-      <c r="B11" s="54"/>
-      <c r="C11" s="214"/>
-      <c r="D11" s="244"/>
+      <c r="B11" s="54" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="244" t="s">
+        <v>71</v>
+      </c>
       <c r="E11" s="64">
         <v>4</v>
       </c>
@@ -4722,9 +4741,15 @@
     </row>
     <row r="12" spans="1:53" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="72"/>
-      <c r="B12" s="37"/>
-      <c r="C12" s="214"/>
-      <c r="D12" s="244"/>
+      <c r="B12" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="C12" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="244" t="s">
+        <v>71</v>
+      </c>
       <c r="E12" s="64">
         <v>5</v>
       </c>
@@ -4863,9 +4888,15 @@
     </row>
     <row r="13" spans="1:53" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="72"/>
-      <c r="B13" s="37"/>
-      <c r="C13" s="214"/>
-      <c r="D13" s="215"/>
+      <c r="B13" s="37" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="215" t="s">
+        <v>71</v>
+      </c>
       <c r="E13" s="64">
         <v>6</v>
       </c>
@@ -5004,8 +5035,12 @@
     </row>
     <row r="14" spans="1:53" s="2" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="30"/>
-      <c r="B14" s="40"/>
-      <c r="C14" s="214"/>
+      <c r="B14" s="40" t="s">
+        <v>69</v>
+      </c>
+      <c r="C14" s="214" t="s">
+        <v>70</v>
+      </c>
       <c r="D14" s="163" t="s">
         <v>77</v>
       </c>
@@ -5147,9 +5182,15 @@
     </row>
     <row r="15" spans="1:53" s="2" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="30"/>
-      <c r="B15" s="29"/>
-      <c r="C15" s="214"/>
-      <c r="D15" s="244"/>
+      <c r="B15" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D15" s="244" t="s">
+        <v>77</v>
+      </c>
       <c r="E15" s="64">
         <v>8</v>
       </c>
@@ -5288,9 +5329,15 @@
     </row>
     <row r="16" spans="1:53" s="2" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="30"/>
-      <c r="B16" s="29"/>
-      <c r="C16" s="214"/>
-      <c r="D16" s="215"/>
+      <c r="B16" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" s="215" t="s">
+        <v>77</v>
+      </c>
       <c r="E16" s="64">
         <v>9</v>
       </c>
@@ -5393,8 +5440,12 @@
     </row>
     <row r="17" spans="1:53" s="2" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="30"/>
-      <c r="B17" s="29"/>
-      <c r="C17" s="214"/>
+      <c r="B17" s="29" t="s">
+        <v>69</v>
+      </c>
+      <c r="C17" s="214" t="s">
+        <v>70</v>
+      </c>
       <c r="D17" s="163" t="s">
         <v>80</v>
       </c>
@@ -5536,8 +5587,12 @@
     </row>
     <row r="18" spans="1:53" s="2" customFormat="1" ht="41.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="30"/>
-      <c r="B18" s="31"/>
-      <c r="C18" s="214"/>
+      <c r="B18" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="C18" s="214" t="s">
+        <v>70</v>
+      </c>
       <c r="D18" s="168" t="s">
         <v>83</v>
       </c>
@@ -5679,8 +5734,12 @@
     </row>
     <row r="19" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="30"/>
-      <c r="B19" s="31"/>
-      <c r="C19" s="214"/>
+      <c r="B19" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="C19" s="214" t="s">
+        <v>70</v>
+      </c>
       <c r="D19" s="163" t="s">
         <v>85</v>
       </c>
@@ -5822,9 +5881,15 @@
     </row>
     <row r="20" spans="1:53" s="2" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="30"/>
-      <c r="B20" s="31"/>
-      <c r="C20" s="237"/>
-      <c r="D20" s="215"/>
+      <c r="B20" s="31" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" s="237" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="215" t="s">
+        <v>85</v>
+      </c>
       <c r="E20" s="64">
         <v>13</v>
       </c>
@@ -5963,7 +6028,9 @@
     </row>
     <row r="21" spans="1:53" s="2" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="30"/>
-      <c r="B21" s="31"/>
+      <c r="B21" s="31" t="s">
+        <v>69</v>
+      </c>
       <c r="C21" s="162" t="s">
         <v>88</v>
       </c>
@@ -6257,9 +6324,15 @@
     </row>
     <row r="23" spans="1:53" s="2" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="30"/>
-      <c r="B23" s="31"/>
-      <c r="C23" s="214"/>
-      <c r="D23" s="244"/>
+      <c r="B23" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C23" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D23" s="244" t="s">
+        <v>94</v>
+      </c>
       <c r="E23" s="64">
         <v>16</v>
       </c>
@@ -6398,9 +6471,15 @@
     </row>
     <row r="24" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="30"/>
-      <c r="B24" s="31"/>
-      <c r="C24" s="214"/>
-      <c r="D24" s="215"/>
+      <c r="B24" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C24" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D24" s="215" t="s">
+        <v>94</v>
+      </c>
       <c r="E24" s="64">
         <v>17</v>
       </c>
@@ -6539,8 +6618,12 @@
     </row>
     <row r="25" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="30"/>
-      <c r="B25" s="31"/>
-      <c r="C25" s="214"/>
+      <c r="B25" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C25" s="214" t="s">
+        <v>70</v>
+      </c>
       <c r="D25" s="172" t="s">
         <v>83</v>
       </c>
@@ -6682,8 +6765,12 @@
     </row>
     <row r="26" spans="1:53" s="2" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="30"/>
-      <c r="B26" s="31"/>
-      <c r="C26" s="214"/>
+      <c r="B26" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C26" s="214" t="s">
+        <v>70</v>
+      </c>
       <c r="D26" s="163" t="s">
         <v>99</v>
       </c>
@@ -6825,9 +6912,15 @@
     </row>
     <row r="27" spans="1:53" s="2" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="30"/>
-      <c r="B27" s="31"/>
-      <c r="C27" s="214"/>
-      <c r="D27" s="244"/>
+      <c r="B27" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C27" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D27" s="244" t="s">
+        <v>99</v>
+      </c>
       <c r="E27" s="64">
         <v>20</v>
       </c>
@@ -6966,9 +7059,15 @@
     </row>
     <row r="28" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="30"/>
-      <c r="B28" s="31"/>
-      <c r="C28" s="214"/>
-      <c r="D28" s="244"/>
+      <c r="B28" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C28" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D28" s="244" t="s">
+        <v>99</v>
+      </c>
       <c r="E28" s="64">
         <v>21</v>
       </c>
@@ -7107,9 +7206,15 @@
     </row>
     <row r="29" spans="1:53" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="30"/>
-      <c r="B29" s="31"/>
-      <c r="C29" s="214"/>
-      <c r="D29" s="244"/>
+      <c r="B29" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C29" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D29" s="244" t="s">
+        <v>99</v>
+      </c>
       <c r="E29" s="64">
         <v>22</v>
       </c>
@@ -7248,9 +7353,15 @@
     </row>
     <row r="30" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="30"/>
-      <c r="B30" s="31"/>
-      <c r="C30" s="237"/>
-      <c r="D30" s="215"/>
+      <c r="B30" s="31" t="s">
+        <v>93</v>
+      </c>
+      <c r="C30" s="237" t="s">
+        <v>70</v>
+      </c>
+      <c r="D30" s="215" t="s">
+        <v>99</v>
+      </c>
       <c r="E30" s="64">
         <v>23</v>
       </c>
@@ -7391,7 +7502,9 @@
     </row>
     <row r="31" spans="1:53" s="1" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="32"/>
-      <c r="B31" s="33"/>
+      <c r="B31" s="33" t="s">
+        <v>93</v>
+      </c>
       <c r="C31" s="264" t="s">
         <v>88</v>
       </c>
@@ -7538,8 +7651,12 @@
     </row>
     <row r="32" spans="1:53" s="1" customFormat="1" ht="55.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="32"/>
-      <c r="B32" s="33"/>
-      <c r="C32" s="265"/>
+      <c r="B32" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="C32" s="265" t="s">
+        <v>88</v>
+      </c>
       <c r="D32" s="176" t="s">
         <v>109</v>
       </c>
@@ -7683,8 +7800,12 @@
     </row>
     <row r="33" spans="1:53" s="1" customFormat="1" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="32"/>
-      <c r="B33" s="33"/>
-      <c r="C33" s="265"/>
+      <c r="B33" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="265" t="s">
+        <v>88</v>
+      </c>
       <c r="D33" s="177" t="s">
         <v>112</v>
       </c>
@@ -7828,8 +7949,12 @@
     </row>
     <row r="34" spans="1:53" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="32"/>
-      <c r="B34" s="33"/>
-      <c r="C34" s="265"/>
+      <c r="B34" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="C34" s="265" t="s">
+        <v>88</v>
+      </c>
       <c r="D34" s="168" t="s">
         <v>114</v>
       </c>
@@ -7971,8 +8096,12 @@
     </row>
     <row r="35" spans="1:53" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="32"/>
-      <c r="B35" s="33"/>
-      <c r="C35" s="265"/>
+      <c r="B35" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="C35" s="265" t="s">
+        <v>88</v>
+      </c>
       <c r="D35" s="163" t="s">
         <v>116</v>
       </c>
@@ -8114,9 +8243,15 @@
     </row>
     <row r="36" spans="1:53" s="1" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="32"/>
-      <c r="B36" s="33"/>
-      <c r="C36" s="266"/>
-      <c r="D36" s="215"/>
+      <c r="B36" s="33" t="s">
+        <v>93</v>
+      </c>
+      <c r="C36" s="266" t="s">
+        <v>88</v>
+      </c>
+      <c r="D36" s="215" t="s">
+        <v>116</v>
+      </c>
       <c r="E36" s="64">
         <v>29</v>
       </c>
@@ -8404,9 +8539,15 @@
     </row>
     <row r="38" spans="1:53" s="1" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="72"/>
-      <c r="B38" s="54"/>
-      <c r="C38" s="214"/>
-      <c r="D38" s="215"/>
+      <c r="B38" s="54" t="s">
+        <v>118</v>
+      </c>
+      <c r="C38" s="214" t="s">
+        <v>119</v>
+      </c>
+      <c r="D38" s="215" t="s">
+        <v>120</v>
+      </c>
       <c r="E38" s="64">
         <v>31</v>
       </c>
@@ -8545,8 +8686,12 @@
     </row>
     <row r="39" spans="1:53" s="1" customFormat="1" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="32"/>
-      <c r="B39" s="59"/>
-      <c r="C39" s="214"/>
+      <c r="B39" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C39" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D39" s="163" t="s">
         <v>124</v>
       </c>
@@ -8688,9 +8833,15 @@
     </row>
     <row r="40" spans="1:53" s="1" customFormat="1" ht="42" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="32"/>
-      <c r="B40" s="59"/>
-      <c r="C40" s="214"/>
-      <c r="D40" s="215"/>
+      <c r="B40" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C40" s="214" t="s">
+        <v>119</v>
+      </c>
+      <c r="D40" s="215" t="s">
+        <v>124</v>
+      </c>
       <c r="E40" s="64">
         <v>33</v>
       </c>
@@ -8829,8 +8980,12 @@
     </row>
     <row r="41" spans="1:53" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="32"/>
-      <c r="B41" s="59"/>
-      <c r="C41" s="214"/>
+      <c r="B41" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C41" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D41" s="241" t="s">
         <v>128</v>
       </c>
@@ -8972,9 +9127,15 @@
     </row>
     <row r="42" spans="1:53" s="1" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="32"/>
-      <c r="B42" s="59"/>
-      <c r="C42" s="214"/>
-      <c r="D42" s="242"/>
+      <c r="B42" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C42" s="214" t="s">
+        <v>119</v>
+      </c>
+      <c r="D42" s="242" t="s">
+        <v>128</v>
+      </c>
       <c r="E42" s="64">
         <v>35</v>
       </c>
@@ -9113,9 +9274,15 @@
     </row>
     <row r="43" spans="1:53" s="1" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="32"/>
-      <c r="B43" s="59"/>
-      <c r="C43" s="214"/>
-      <c r="D43" s="243"/>
+      <c r="B43" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C43" s="214" t="s">
+        <v>119</v>
+      </c>
+      <c r="D43" s="243" t="s">
+        <v>128</v>
+      </c>
       <c r="E43" s="64">
         <v>36</v>
       </c>
@@ -9254,8 +9421,12 @@
     </row>
     <row r="44" spans="1:53" s="1" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="32"/>
-      <c r="B44" s="59"/>
-      <c r="C44" s="214"/>
+      <c r="B44" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C44" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D44" s="175" t="s">
         <v>133</v>
       </c>
@@ -9399,8 +9570,12 @@
     </row>
     <row r="45" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="32"/>
-      <c r="B45" s="59"/>
-      <c r="C45" s="214"/>
+      <c r="B45" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C45" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D45" s="175" t="s">
         <v>135</v>
       </c>
@@ -9544,8 +9719,12 @@
     </row>
     <row r="46" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="32"/>
-      <c r="B46" s="59"/>
-      <c r="C46" s="214"/>
+      <c r="B46" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C46" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D46" s="175" t="s">
         <v>137</v>
       </c>
@@ -9689,8 +9868,12 @@
     </row>
     <row r="47" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="32"/>
-      <c r="B47" s="124"/>
-      <c r="C47" s="214"/>
+      <c r="B47" s="124" t="s">
+        <v>118</v>
+      </c>
+      <c r="C47" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D47" s="175" t="s">
         <v>139</v>
       </c>
@@ -9834,8 +10017,12 @@
     </row>
     <row r="48" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="32"/>
-      <c r="B48" s="59"/>
-      <c r="C48" s="214"/>
+      <c r="B48" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C48" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D48" s="238" t="s">
         <v>141</v>
       </c>
@@ -9979,9 +10166,15 @@
     </row>
     <row r="49" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="32"/>
-      <c r="B49" s="59"/>
-      <c r="C49" s="214"/>
-      <c r="D49" s="239"/>
+      <c r="B49" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C49" s="214" t="s">
+        <v>119</v>
+      </c>
+      <c r="D49" s="239" t="s">
+        <v>141</v>
+      </c>
       <c r="E49" s="64">
         <v>42</v>
       </c>
@@ -10122,9 +10315,15 @@
     </row>
     <row r="50" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="32"/>
-      <c r="B50" s="59"/>
-      <c r="C50" s="237"/>
-      <c r="D50" s="240"/>
+      <c r="B50" s="59" t="s">
+        <v>118</v>
+      </c>
+      <c r="C50" s="237" t="s">
+        <v>119</v>
+      </c>
+      <c r="D50" s="240" t="s">
+        <v>141</v>
+      </c>
       <c r="E50" s="64">
         <v>43</v>
       </c>
@@ -10265,7 +10464,9 @@
     </row>
     <row r="51" spans="1:53" s="1" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="32"/>
-      <c r="B51" s="59"/>
+      <c r="B51" s="59" t="s">
+        <v>118</v>
+      </c>
       <c r="C51" s="188" t="s">
         <v>145</v>
       </c>
@@ -10559,9 +10760,15 @@
     </row>
     <row r="53" spans="1:53" s="2" customFormat="1" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="35"/>
-      <c r="B53" s="36"/>
-      <c r="C53" s="214"/>
-      <c r="D53" s="215"/>
+      <c r="B53" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="C53" s="214" t="s">
+        <v>88</v>
+      </c>
+      <c r="D53" s="215" t="s">
+        <v>109</v>
+      </c>
       <c r="E53" s="64">
         <v>46</v>
       </c>
@@ -10702,8 +10909,12 @@
     </row>
     <row r="54" spans="1:53" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="38"/>
-      <c r="B54" s="37"/>
-      <c r="C54" s="214"/>
+      <c r="B54" s="37" t="s">
+        <v>148</v>
+      </c>
+      <c r="C54" s="214" t="s">
+        <v>88</v>
+      </c>
       <c r="D54" s="163" t="s">
         <v>112</v>
       </c>
@@ -10845,9 +11056,15 @@
     </row>
     <row r="55" spans="1:53" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="38"/>
-      <c r="B55" s="37"/>
-      <c r="C55" s="214"/>
-      <c r="D55" s="215"/>
+      <c r="B55" s="37" t="s">
+        <v>148</v>
+      </c>
+      <c r="C55" s="214" t="s">
+        <v>88</v>
+      </c>
+      <c r="D55" s="215" t="s">
+        <v>112</v>
+      </c>
       <c r="E55" s="64">
         <v>48</v>
       </c>
@@ -10988,8 +11205,12 @@
     </row>
     <row r="56" spans="1:53" s="2" customFormat="1" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="39"/>
-      <c r="B56" s="40"/>
-      <c r="C56" s="214"/>
+      <c r="B56" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="C56" s="214" t="s">
+        <v>88</v>
+      </c>
       <c r="D56" s="163" t="s">
         <v>114</v>
       </c>
@@ -11133,9 +11354,15 @@
     </row>
     <row r="57" spans="1:53" s="2" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="39"/>
-      <c r="B57" s="40"/>
-      <c r="C57" s="214"/>
-      <c r="D57" s="215"/>
+      <c r="B57" s="40" t="s">
+        <v>148</v>
+      </c>
+      <c r="C57" s="214" t="s">
+        <v>88</v>
+      </c>
+      <c r="D57" s="215" t="s">
+        <v>114</v>
+      </c>
       <c r="E57" s="64">
         <v>50</v>
       </c>
@@ -11274,8 +11501,12 @@
     </row>
     <row r="58" spans="1:53" s="2" customFormat="1" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="39"/>
-      <c r="B58" s="55"/>
-      <c r="C58" s="237"/>
+      <c r="B58" s="55" t="s">
+        <v>148</v>
+      </c>
+      <c r="C58" s="237" t="s">
+        <v>88</v>
+      </c>
       <c r="D58" s="163" t="s">
         <v>116</v>
       </c>
@@ -11566,9 +11797,15 @@
     </row>
     <row r="60" spans="1:53" s="1" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="28"/>
-      <c r="B60" s="36"/>
-      <c r="C60" s="214"/>
-      <c r="D60" s="239"/>
+      <c r="B60" s="36" t="s">
+        <v>160</v>
+      </c>
+      <c r="C60" s="214" t="s">
+        <v>161</v>
+      </c>
+      <c r="D60" s="239" t="s">
+        <v>162</v>
+      </c>
       <c r="E60" s="64">
         <v>53</v>
       </c>
@@ -11707,9 +11944,15 @@
     </row>
     <row r="61" spans="1:53" s="2" customFormat="1" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="153"/>
-      <c r="B61" s="154"/>
-      <c r="C61" s="214"/>
-      <c r="D61" s="239"/>
+      <c r="B61" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C61" s="214" t="s">
+        <v>161</v>
+      </c>
+      <c r="D61" s="239" t="s">
+        <v>162</v>
+      </c>
       <c r="E61" s="64">
         <v>54</v>
       </c>
@@ -11848,9 +12091,15 @@
     </row>
     <row r="62" spans="1:53" s="2" customFormat="1" ht="57" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="153"/>
-      <c r="B62" s="154"/>
-      <c r="C62" s="214"/>
-      <c r="D62" s="239"/>
+      <c r="B62" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C62" s="214" t="s">
+        <v>161</v>
+      </c>
+      <c r="D62" s="239" t="s">
+        <v>162</v>
+      </c>
       <c r="E62" s="64">
         <v>55</v>
       </c>
@@ -11989,9 +12238,15 @@
     </row>
     <row r="63" spans="1:53" s="2" customFormat="1" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="153"/>
-      <c r="B63" s="154"/>
-      <c r="C63" s="214"/>
-      <c r="D63" s="239"/>
+      <c r="B63" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C63" s="214" t="s">
+        <v>161</v>
+      </c>
+      <c r="D63" s="239" t="s">
+        <v>162</v>
+      </c>
       <c r="E63" s="64">
         <v>56</v>
       </c>
@@ -12130,9 +12385,15 @@
     </row>
     <row r="64" spans="1:53" s="2" customFormat="1" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="153"/>
-      <c r="B64" s="154"/>
-      <c r="C64" s="237"/>
-      <c r="D64" s="240"/>
+      <c r="B64" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C64" s="237" t="s">
+        <v>161</v>
+      </c>
+      <c r="D64" s="240" t="s">
+        <v>162</v>
+      </c>
       <c r="E64" s="64">
         <v>57</v>
       </c>
@@ -12271,7 +12532,9 @@
     </row>
     <row r="65" spans="1:53" s="2" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="153"/>
-      <c r="B65" s="154"/>
+      <c r="B65" s="154" t="s">
+        <v>160</v>
+      </c>
       <c r="C65" s="162" t="s">
         <v>56</v>
       </c>
@@ -12416,9 +12679,15 @@
     </row>
     <row r="66" spans="1:53" s="2" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="153"/>
-      <c r="B66" s="154"/>
-      <c r="C66" s="214"/>
-      <c r="D66" s="244"/>
+      <c r="B66" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C66" s="214" t="s">
+        <v>56</v>
+      </c>
+      <c r="D66" s="244" t="s">
+        <v>57</v>
+      </c>
       <c r="E66" s="64">
         <v>59</v>
       </c>
@@ -12559,9 +12828,15 @@
     </row>
     <row r="67" spans="1:53" s="2" customFormat="1" ht="54" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="153"/>
-      <c r="B67" s="154"/>
-      <c r="C67" s="214"/>
-      <c r="D67" s="215"/>
+      <c r="B67" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C67" s="214" t="s">
+        <v>56</v>
+      </c>
+      <c r="D67" s="215" t="s">
+        <v>57</v>
+      </c>
       <c r="E67" s="64">
         <v>60</v>
       </c>
@@ -12700,8 +12975,12 @@
     </row>
     <row r="68" spans="1:53" s="2" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="153"/>
-      <c r="B68" s="154"/>
-      <c r="C68" s="214"/>
+      <c r="B68" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C68" s="214" t="s">
+        <v>56</v>
+      </c>
       <c r="D68" s="163" t="s">
         <v>174</v>
       </c>
@@ -12843,9 +13122,15 @@
     </row>
     <row r="69" spans="1:53" s="2" customFormat="1" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="153"/>
-      <c r="B69" s="154"/>
-      <c r="C69" s="237"/>
-      <c r="D69" s="215"/>
+      <c r="B69" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C69" s="237" t="s">
+        <v>56</v>
+      </c>
+      <c r="D69" s="215" t="s">
+        <v>174</v>
+      </c>
       <c r="E69" s="64">
         <v>62</v>
       </c>
@@ -12984,7 +13269,9 @@
     </row>
     <row r="70" spans="1:53" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="153"/>
-      <c r="B70" s="154"/>
+      <c r="B70" s="154" t="s">
+        <v>160</v>
+      </c>
       <c r="C70" s="162" t="s">
         <v>119</v>
       </c>
@@ -13129,8 +13416,12 @@
     </row>
     <row r="71" spans="1:53" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="153"/>
-      <c r="B71" s="154"/>
-      <c r="C71" s="214"/>
+      <c r="B71" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C71" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D71" s="176" t="s">
         <v>128</v>
       </c>
@@ -13272,8 +13563,12 @@
     </row>
     <row r="72" spans="1:53" s="2" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="153"/>
-      <c r="B72" s="154"/>
-      <c r="C72" s="214"/>
+      <c r="B72" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C72" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D72" s="176" t="s">
         <v>180</v>
       </c>
@@ -13415,8 +13710,12 @@
     </row>
     <row r="73" spans="1:53" s="2" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="153"/>
-      <c r="B73" s="154"/>
-      <c r="C73" s="214"/>
+      <c r="B73" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C73" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D73" s="175" t="s">
         <v>133</v>
       </c>
@@ -13558,8 +13857,12 @@
     </row>
     <row r="74" spans="1:53" s="2" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="153"/>
-      <c r="B74" s="154"/>
-      <c r="C74" s="214"/>
+      <c r="B74" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C74" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D74" s="175" t="s">
         <v>135</v>
       </c>
@@ -13701,8 +14004,12 @@
     </row>
     <row r="75" spans="1:53" s="2" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="153"/>
-      <c r="B75" s="154"/>
-      <c r="C75" s="214"/>
+      <c r="B75" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C75" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D75" s="175" t="s">
         <v>137</v>
       </c>
@@ -13844,8 +14151,12 @@
     </row>
     <row r="76" spans="1:53" s="2" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="153"/>
-      <c r="B76" s="154"/>
-      <c r="C76" s="214"/>
+      <c r="B76" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C76" s="214" t="s">
+        <v>119</v>
+      </c>
       <c r="D76" s="175" t="s">
         <v>139</v>
       </c>
@@ -13987,8 +14298,12 @@
     </row>
     <row r="77" spans="1:53" s="2" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="153"/>
-      <c r="B77" s="154"/>
-      <c r="C77" s="237"/>
+      <c r="B77" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C77" s="237" t="s">
+        <v>119</v>
+      </c>
       <c r="D77" s="163" t="s">
         <v>124</v>
       </c>
@@ -14130,7 +14445,9 @@
     </row>
     <row r="78" spans="1:53" s="2" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="153"/>
-      <c r="B78" s="154"/>
+      <c r="B78" s="154" t="s">
+        <v>160</v>
+      </c>
       <c r="C78" s="162" t="s">
         <v>184</v>
       </c>
@@ -14275,9 +14592,15 @@
     </row>
     <row r="79" spans="1:53" s="2" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="153"/>
-      <c r="B79" s="154"/>
-      <c r="C79" s="214"/>
-      <c r="D79" s="215"/>
+      <c r="B79" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C79" s="214" t="s">
+        <v>184</v>
+      </c>
+      <c r="D79" s="215" t="s">
+        <v>185</v>
+      </c>
       <c r="E79" s="64">
         <v>72</v>
       </c>
@@ -14416,8 +14739,12 @@
     </row>
     <row r="80" spans="1:53" s="2" customFormat="1" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="153"/>
-      <c r="B80" s="154"/>
-      <c r="C80" s="214"/>
+      <c r="B80" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C80" s="214" t="s">
+        <v>184</v>
+      </c>
       <c r="D80" s="163" t="s">
         <v>188</v>
       </c>
@@ -14559,9 +14886,15 @@
     </row>
     <row r="81" spans="1:53" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="153"/>
-      <c r="B81" s="154"/>
-      <c r="C81" s="214"/>
-      <c r="D81" s="244"/>
+      <c r="B81" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C81" s="214" t="s">
+        <v>184</v>
+      </c>
+      <c r="D81" s="244" t="s">
+        <v>188</v>
+      </c>
       <c r="E81" s="64">
         <v>74</v>
       </c>
@@ -14700,9 +15033,15 @@
     </row>
     <row r="82" spans="1:53" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="153"/>
-      <c r="B82" s="153"/>
-      <c r="C82" s="214"/>
-      <c r="D82" s="244"/>
+      <c r="B82" s="153" t="s">
+        <v>160</v>
+      </c>
+      <c r="C82" s="214" t="s">
+        <v>184</v>
+      </c>
+      <c r="D82" s="244" t="s">
+        <v>188</v>
+      </c>
       <c r="E82" s="64">
         <v>75</v>
       </c>
@@ -14841,9 +15180,15 @@
     </row>
     <row r="83" spans="1:53" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="153"/>
-      <c r="B83" s="153"/>
-      <c r="C83" s="237"/>
-      <c r="D83" s="215"/>
+      <c r="B83" s="153" t="s">
+        <v>160</v>
+      </c>
+      <c r="C83" s="237" t="s">
+        <v>184</v>
+      </c>
+      <c r="D83" s="215" t="s">
+        <v>188</v>
+      </c>
       <c r="E83" s="64">
         <v>76</v>
       </c>
@@ -14982,7 +15327,9 @@
     </row>
     <row r="84" spans="1:53" s="2" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="153"/>
-      <c r="B84" s="153"/>
+      <c r="B84" s="153" t="s">
+        <v>160</v>
+      </c>
       <c r="C84" s="162" t="s">
         <v>70</v>
       </c>
@@ -15127,9 +15474,15 @@
     </row>
     <row r="85" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="154"/>
-      <c r="B85" s="155"/>
-      <c r="C85" s="214"/>
-      <c r="D85" s="215"/>
+      <c r="B85" s="155" t="s">
+        <v>160</v>
+      </c>
+      <c r="C85" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D85" s="215" t="s">
+        <v>193</v>
+      </c>
       <c r="E85" s="64">
         <v>78</v>
       </c>
@@ -15268,8 +15621,12 @@
     </row>
     <row r="86" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="156"/>
-      <c r="B86" s="155"/>
-      <c r="C86" s="214"/>
+      <c r="B86" s="155" t="s">
+        <v>160</v>
+      </c>
+      <c r="C86" s="214" t="s">
+        <v>70</v>
+      </c>
       <c r="D86" s="168" t="s">
         <v>99</v>
       </c>
@@ -15411,8 +15768,12 @@
     </row>
     <row r="87" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="156"/>
-      <c r="B87" s="155"/>
-      <c r="C87" s="237"/>
+      <c r="B87" s="155" t="s">
+        <v>160</v>
+      </c>
+      <c r="C87" s="237" t="s">
+        <v>70</v>
+      </c>
       <c r="D87" s="168" t="s">
         <v>83</v>
       </c>
@@ -15554,7 +15915,9 @@
     </row>
     <row r="88" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="154"/>
-      <c r="B88" s="155"/>
+      <c r="B88" s="155" t="s">
+        <v>160</v>
+      </c>
       <c r="C88" s="162" t="s">
         <v>88</v>
       </c>
@@ -15699,8 +16062,12 @@
     </row>
     <row r="89" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="156"/>
-      <c r="B89" s="155"/>
-      <c r="C89" s="214"/>
+      <c r="B89" s="155" t="s">
+        <v>160</v>
+      </c>
+      <c r="C89" s="214" t="s">
+        <v>88</v>
+      </c>
       <c r="D89" s="163" t="s">
         <v>114</v>
       </c>
@@ -15842,9 +16209,15 @@
     </row>
     <row r="90" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="156"/>
-      <c r="B90" s="155"/>
-      <c r="C90" s="214"/>
-      <c r="D90" s="215"/>
+      <c r="B90" s="155" t="s">
+        <v>160</v>
+      </c>
+      <c r="C90" s="214" t="s">
+        <v>88</v>
+      </c>
+      <c r="D90" s="215" t="s">
+        <v>114</v>
+      </c>
       <c r="E90" s="64">
         <v>83</v>
       </c>
@@ -15983,8 +16356,12 @@
     </row>
     <row r="91" spans="1:53" s="2" customFormat="1" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="154"/>
-      <c r="B91" s="155"/>
-      <c r="C91" s="214"/>
+      <c r="B91" s="155" t="s">
+        <v>160</v>
+      </c>
+      <c r="C91" s="214" t="s">
+        <v>88</v>
+      </c>
       <c r="D91" s="175" t="s">
         <v>116</v>
       </c>
@@ -16126,8 +16503,12 @@
     </row>
     <row r="92" spans="1:53" s="2" customFormat="1" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="155"/>
-      <c r="B92" s="154"/>
-      <c r="C92" s="214"/>
+      <c r="B92" s="154" t="s">
+        <v>160</v>
+      </c>
+      <c r="C92" s="214" t="s">
+        <v>88</v>
+      </c>
       <c r="D92" s="175" t="s">
         <v>205</v>
       </c>
@@ -16271,8 +16652,12 @@
     </row>
     <row r="93" spans="1:53" s="2" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="142"/>
-      <c r="B93" s="155"/>
-      <c r="C93" s="237"/>
+      <c r="B93" s="155" t="s">
+        <v>160</v>
+      </c>
+      <c r="C93" s="237" t="s">
+        <v>88</v>
+      </c>
       <c r="D93" s="202" t="s">
         <v>207</v>
       </c>
@@ -16563,8 +16948,12 @@
     </row>
     <row r="95" spans="1:53" s="1" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="105"/>
-      <c r="B95" s="36"/>
-      <c r="C95" s="265"/>
+      <c r="B95" s="36" t="s">
+        <v>204</v>
+      </c>
+      <c r="C95" s="265" t="s">
+        <v>88</v>
+      </c>
       <c r="D95" s="238" t="s">
         <v>204</v>
       </c>
@@ -16706,9 +17095,15 @@
     </row>
     <row r="96" spans="1:53" s="1" customFormat="1" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="34"/>
-      <c r="B96" s="157"/>
-      <c r="C96" s="265"/>
-      <c r="D96" s="239"/>
+      <c r="B96" s="157" t="s">
+        <v>204</v>
+      </c>
+      <c r="C96" s="265" t="s">
+        <v>88</v>
+      </c>
+      <c r="D96" s="239" t="s">
+        <v>204</v>
+      </c>
       <c r="E96" s="64">
         <v>89</v>
       </c>
@@ -16847,9 +17242,15 @@
     </row>
     <row r="97" spans="1:53" s="1" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="34"/>
-      <c r="B97" s="157"/>
-      <c r="C97" s="265"/>
-      <c r="D97" s="239"/>
+      <c r="B97" s="157" t="s">
+        <v>204</v>
+      </c>
+      <c r="C97" s="265" t="s">
+        <v>88</v>
+      </c>
+      <c r="D97" s="239" t="s">
+        <v>204</v>
+      </c>
       <c r="E97" s="64">
         <v>90</v>
       </c>
@@ -16988,9 +17389,15 @@
     </row>
     <row r="98" spans="1:53" s="1" customFormat="1" ht="34.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="34"/>
-      <c r="B98" s="157"/>
-      <c r="C98" s="265"/>
-      <c r="D98" s="240"/>
+      <c r="B98" s="157" t="s">
+        <v>204</v>
+      </c>
+      <c r="C98" s="265" t="s">
+        <v>88</v>
+      </c>
+      <c r="D98" s="240" t="s">
+        <v>204</v>
+      </c>
       <c r="E98" s="64">
         <v>91</v>
       </c>
@@ -17129,8 +17536,12 @@
     </row>
     <row r="99" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="34"/>
-      <c r="B99" s="157"/>
-      <c r="C99" s="267"/>
+      <c r="B99" s="157" t="s">
+        <v>204</v>
+      </c>
+      <c r="C99" s="267" t="s">
+        <v>88</v>
+      </c>
       <c r="D99" s="163" t="s">
         <v>215</v>
       </c>
@@ -17272,9 +17683,15 @@
     </row>
     <row r="100" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="34"/>
-      <c r="B100" s="157"/>
-      <c r="C100" s="267"/>
-      <c r="D100" s="215"/>
+      <c r="B100" s="157" t="s">
+        <v>204</v>
+      </c>
+      <c r="C100" s="267" t="s">
+        <v>88</v>
+      </c>
+      <c r="D100" s="215" t="s">
+        <v>215</v>
+      </c>
       <c r="E100" s="64">
         <v>93</v>
       </c>
@@ -17413,8 +17830,12 @@
     </row>
     <row r="101" spans="1:53" s="1" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="34"/>
-      <c r="B101" s="158"/>
-      <c r="C101" s="266"/>
+      <c r="B101" s="158" t="s">
+        <v>204</v>
+      </c>
+      <c r="C101" s="266" t="s">
+        <v>88</v>
+      </c>
       <c r="D101" s="175" t="s">
         <v>89</v>
       </c>
@@ -17705,7 +18126,9 @@
     </row>
     <row r="103" spans="1:53" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="75"/>
-      <c r="B103" s="54"/>
+      <c r="B103" s="54" t="s">
+        <v>219</v>
+      </c>
       <c r="C103" s="162" t="s">
         <v>70</v>
       </c>
@@ -17846,9 +18269,15 @@
     </row>
     <row r="104" spans="1:53" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="75"/>
-      <c r="B104" s="54"/>
-      <c r="C104" s="214"/>
-      <c r="D104" s="244"/>
+      <c r="B104" s="54" t="s">
+        <v>219</v>
+      </c>
+      <c r="C104" s="214" t="s">
+        <v>70</v>
+      </c>
+      <c r="D104" s="244" t="s">
+        <v>258</v>
+      </c>
       <c r="E104" s="64">
         <v>97</v>
       </c>
@@ -17986,9 +18415,15 @@
     </row>
     <row r="105" spans="1:53" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="75"/>
-      <c r="B105" s="54"/>
-      <c r="C105" s="237"/>
-      <c r="D105" s="215"/>
+      <c r="B105" s="54" t="s">
+        <v>219</v>
+      </c>
+      <c r="C105" s="237" t="s">
+        <v>70</v>
+      </c>
+      <c r="D105" s="215" t="s">
+        <v>258</v>
+      </c>
       <c r="E105" s="64">
         <v>98</v>
       </c>
@@ -18123,7 +18558,9 @@
     </row>
     <row r="106" spans="1:53" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="76"/>
-      <c r="B106" s="54"/>
+      <c r="B106" s="54" t="s">
+        <v>219</v>
+      </c>
       <c r="C106" s="211" t="s">
         <v>145</v>
       </c>

</xml_diff>